<commit_message>
Updated timline theme and added sample input data
</commit_message>
<xml_diff>
--- a/TaskInfo.xlsx
+++ b/TaskInfo.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="50">
   <si>
     <t>EpicNo</t>
   </si>
@@ -39,10 +39,22 @@
     <t>Amey</t>
   </si>
   <si>
+    <t>[QA]Story1</t>
+  </si>
+  <si>
+    <t>QA1</t>
+  </si>
+  <si>
     <t>Story2</t>
   </si>
   <si>
     <t>Shreya</t>
+  </si>
+  <si>
+    <t>[QA]Story2</t>
+  </si>
+  <si>
+    <t>QA2</t>
   </si>
   <si>
     <t>Story3</t>
@@ -51,10 +63,16 @@
     <t>Rakesh</t>
   </si>
   <si>
+    <t>[QA]Story3</t>
+  </si>
+  <si>
     <t>Story4</t>
   </si>
   <si>
     <t>Aditi</t>
+  </si>
+  <si>
+    <t>[QA]Story4</t>
   </si>
   <si>
     <t>Story5</t>
@@ -63,79 +81,67 @@
     <t>Shaina</t>
   </si>
   <si>
+    <t>[QA]Story5</t>
+  </si>
+  <si>
     <t>Story6</t>
+  </si>
+  <si>
+    <t>[QA]Story6</t>
   </si>
   <si>
     <t>Story7</t>
   </si>
   <si>
+    <t>[QA]Story7</t>
+  </si>
+  <si>
     <t>Story8</t>
+  </si>
+  <si>
+    <t>[QA]Story8</t>
   </si>
   <si>
     <t>Story9</t>
   </si>
   <si>
+    <t>[QA]Story9</t>
+  </si>
+  <si>
     <t>Story10</t>
+  </si>
+  <si>
+    <t>[QA]Story10</t>
   </si>
   <si>
     <t>Story11</t>
   </si>
   <si>
+    <t>[QA]Story11</t>
+  </si>
+  <si>
     <t>Story12</t>
+  </si>
+  <si>
+    <t>[QA]Story12</t>
   </si>
   <si>
     <t>Story13</t>
   </si>
   <si>
+    <t>[QA]Story13</t>
+  </si>
+  <si>
     <t>Story14</t>
+  </si>
+  <si>
+    <t>[QA]Story14</t>
   </si>
   <si>
     <t>Story15</t>
   </si>
   <si>
-    <t>Story16</t>
-  </si>
-  <si>
-    <t>Story17</t>
-  </si>
-  <si>
-    <t>Story18</t>
-  </si>
-  <si>
-    <t>Story19</t>
-  </si>
-  <si>
-    <t>Story20</t>
-  </si>
-  <si>
-    <t>Story21</t>
-  </si>
-  <si>
-    <t>Story22</t>
-  </si>
-  <si>
-    <t>Story23</t>
-  </si>
-  <si>
-    <t>Story24</t>
-  </si>
-  <si>
-    <t>Story25</t>
-  </si>
-  <si>
-    <t>Story26</t>
-  </si>
-  <si>
-    <t>Story27</t>
-  </si>
-  <si>
-    <t>Story28</t>
-  </si>
-  <si>
-    <t>Story29</t>
-  </si>
-  <si>
-    <t>Story30</t>
+    <t>[QA]Story15</t>
   </si>
   <si>
     <t>Player</t>
@@ -169,7 +175,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -188,6 +194,12 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -245,10 +257,10 @@
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -268,10 +280,10 @@
     <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -612,13 +624,13 @@
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
       <c r="A1" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D1" s="12"/>
       <c r="E1" s="12"/>
@@ -646,7 +658,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
       <c r="A2" s="12" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B2" s="16">
         <v>46027</v>
@@ -680,7 +692,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
       <c r="A3" s="12" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B3" s="16">
         <v>46048</v>
@@ -714,7 +726,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
       <c r="A4" s="12" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B4" s="16">
         <v>46097</v>
@@ -28653,10 +28665,10 @@
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
@@ -28677,7 +28689,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
       <c r="A4" s="12" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B4" s="13">
         <v>46096</v>
@@ -28685,7 +28697,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
       <c r="A5" s="12" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B5" s="13">
         <v>46113</v>
@@ -28693,7 +28705,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
       <c r="A6" s="12" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B6" s="13">
         <v>46093</v>
@@ -28701,7 +28713,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
       <c r="A7" s="12" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B7" s="13">
         <v>46114</v>
@@ -28709,7 +28721,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
       <c r="A8" s="12" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B8" s="13">
         <v>46103</v>
@@ -28717,7 +28729,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
       <c r="A9" s="12" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B9" s="13">
         <v>46117</v>
@@ -28725,7 +28737,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25">
       <c r="A10" s="12" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B10" s="13">
         <v>46089</v>
@@ -28733,7 +28745,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25">
       <c r="A11" s="12" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B11" s="13">
         <v>46116</v>
@@ -28759,7 +28771,7 @@
     <col min="5" max="5" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -28776,7 +28788,7 @@
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -28793,7 +28805,7 @@
         <v>46087.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -28804,13 +28816,13 @@
         <v>8</v>
       </c>
       <c r="D3" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E3" s="7">
         <v>46087.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="5">
         <v>1</v>
       </c>
@@ -28821,13 +28833,13 @@
         <v>10</v>
       </c>
       <c r="D4" s="5">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E4" s="7">
-        <v>46118.229166666664</v>
+        <v>46087.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -28838,15 +28850,15 @@
         <v>12</v>
       </c>
       <c r="D5" s="5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E5" s="7">
-        <v>46118.229166666664</v>
+        <v>46087.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>13</v>
@@ -28855,222 +28867,222 @@
         <v>14</v>
       </c>
       <c r="D6" s="5">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E6" s="7">
-        <v>46087.229166666664</v>
+        <v>46118.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D7" s="5">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E7" s="7">
         <v>46118.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D8" s="5">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="E8" s="7">
-        <v>46087.229166666664</v>
+        <v>46118.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D9" s="5">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E9" s="7">
         <v>46118.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D10" s="5">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E10" s="7">
         <v>46087.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D11" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11" s="7">
-        <v>46118.229166666664</v>
+        <v>46087.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D12" s="5">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E12" s="7">
-        <v>46087.229166666664</v>
+        <v>46118.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D13" s="5">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E13" s="7">
         <v>46118.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D14" s="5">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="E14" s="7">
         <v>46087.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D15" s="5">
         <v>5</v>
       </c>
       <c r="E15" s="7">
+        <v>46087.229166666664</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+      <c r="A16" s="5">
+        <v>2</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="5">
+        <v>5</v>
+      </c>
+      <c r="E16" s="7">
         <v>46118.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
-      <c r="A16" s="5">
-        <v>4</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D16" s="5">
-        <v>8</v>
-      </c>
-      <c r="E16" s="7">
-        <v>46087.229166666664</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D17" s="5">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="E17" s="7">
         <v>46118.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D18" s="5">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E18" s="7">
         <v>46087.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>8</v>
@@ -29079,106 +29091,106 @@
         <v>3</v>
       </c>
       <c r="E19" s="7">
+        <v>46087.229166666664</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+      <c r="A20" s="5">
+        <v>3</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" s="5">
+        <v>3</v>
+      </c>
+      <c r="E20" s="7">
         <v>46118.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="17.25">
-      <c r="A20" s="5">
-        <v>5</v>
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+      <c r="A21" s="5">
+        <v>3</v>
       </c>
-      <c r="B20" s="6" t="s">
-        <v>28</v>
+      <c r="B21" s="6" t="s">
+        <v>31</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C21" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="5">
-        <v>8</v>
-      </c>
-      <c r="E20" s="7">
-        <v>46087.229166666664</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="17.25">
-      <c r="A21" s="5">
-        <v>5</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>14</v>
-      </c>
       <c r="D21" s="5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E21" s="7">
         <v>46118.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="5">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D22" s="5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E22" s="7">
         <v>46087.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="5">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D23" s="5">
+        <v>2</v>
+      </c>
+      <c r="E23" s="7">
+        <v>46087.229166666664</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+      <c r="A24" s="5">
+        <v>3</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="5">
         <v>8</v>
       </c>
-      <c r="E23" s="7">
+      <c r="E24" s="7">
         <v>46118.229166666664</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="17.25">
-      <c r="A24" s="5">
-        <v>6</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D24" s="5">
-        <v>13</v>
-      </c>
-      <c r="E24" s="7">
-        <v>46087.229166666664</v>
-      </c>
-    </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="17.25">
       <c r="A25" s="5">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D25" s="5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E25" s="7">
         <v>46118.229166666664</v>
@@ -29186,13 +29198,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="17.25">
       <c r="A26" s="5">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D26" s="5">
         <v>3</v>
@@ -29203,50 +29215,50 @@
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="17.25">
       <c r="A27" s="5">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D27" s="5">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E27" s="7">
-        <v>46118.229166666664</v>
+        <v>46087.229166666664</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="17.25">
       <c r="A28" s="5">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D28" s="5">
         <v>5</v>
       </c>
       <c r="E28" s="7">
-        <v>46087.229166666664</v>
+        <v>46118.229166666664</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="17.25">
       <c r="A29" s="5">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D29" s="5">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="E29" s="7">
         <v>46118.229166666664</v>
@@ -29254,13 +29266,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="17.25">
       <c r="A30" s="5">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D30" s="5">
         <v>8</v>
@@ -29271,19 +29283,19 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="17.25">
       <c r="A31" s="5">
+        <v>4</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C31" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B31" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>14</v>
-      </c>
       <c r="D31" s="5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E31" s="7">
-        <v>46118.229166666664</v>
+        <v>46087.229166666664</v>
       </c>
     </row>
   </sheetData>

</xml_diff>